<commit_message>
use of meds fix
</commit_message>
<xml_diff>
--- a/SurveyQuestions/outputs/hms_question_score.xlsx
+++ b/SurveyQuestions/outputs/hms_question_score.xlsx
@@ -5273,12 +5273,12 @@
       <c r="P37" s="2" t="inlineStr"/>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
+          <t>Display if "8=No, none of these" is not selected for "In the past 12 months have you taken any of the following types of prescription medications?" Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
+          <t>Display if "8=No, none of these" is not selected for "In the past 12 months have you taken any of the following types of prescription medications?" Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
         </is>
       </c>
     </row>
@@ -5543,12 +5543,12 @@
       <c r="P42" s="2" t="inlineStr"/>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
+          <t>Display if "8=No, none of these" is not selected for "In the past 12 months have you taken any of the following types of prescription medications?" Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
         </is>
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
+          <t>Display if "8=No, none of these" is not selected for "In the past 12 months have you taken any of the following types of prescription medications?" Pipe in selected options from: “In the past 12 months have you taken any of the following types of prescription medications?”</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
made FE qn matrix
</commit_message>
<xml_diff>
--- a/SurveyQuestions/outputs/hms_question_score.xlsx
+++ b/SurveyQuestions/outputs/hms_question_score.xlsx
@@ -1718,7 +1718,7 @@
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1=Yes 0=No</t>
+          <t>0=No 1=Yes</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -9534,7 +9534,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Likert (6-point)</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -9552,11 +9552,11 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -9569,14 +9569,18 @@
         </is>
       </c>
       <c r="O10" s="2" t="n">
-        <v>0.597</v>
+        <v>0.647</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr"/>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix table with 3 statements.</t>
+        </is>
+      </c>
       <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
dry run fix #1
</commit_message>
<xml_diff>
--- a/SurveyQuestions/outputs/hms_question_score.xlsx
+++ b/SurveyQuestions/outputs/hms_question_score.xlsx
@@ -1627,7 +1627,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Please answer the following questions as honestly as possible. Do you often feel the desire to eat when you are emotionally upset or stressed? Do you often feel that you can't control what or how much you eat? Do you sometimes make yourself throw up (vomit) to control your weight? Are you often preoccupied with a desire to be thinner? Do you believe yourself to be fat when others say you are thin?</t>
+          <t>Please answer the following questions as honestly as possible. 1. Do you often feel the desire to eat when you are emotionally upset or stressed? 2. Do you often feel that you can't control what or how much you eat? 3. Do you sometimes make yourself throw up (vomit) to control your weight? 4. Are you often preoccupied with a desire to be thinner? 5. Do you believe yourself to be fat when others say you are thin?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1643,15 +1643,15 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Matrix</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>68.06999999999999</v>
+        <v>74.13</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1661,11 +1661,11 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="O10" s="2" t="n">
-        <v>0.397</v>
+        <v>0.435</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -1687,14 +1687,10 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Included if ‘Eating and Body Image’ module not selected SDE (Maguen et al., 2018)</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>Included if ‘Eating and Body Image’ module not selected SDE (Maguen et al., 2018)</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Matrix </t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2170,7 +2166,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>1=0 times 2=1 time 3=2 times 4=3 to 5 times 5=6 to 9 times 6=10 or more times 7=Don’t know</t>
+          <t xml:space="preserve">1=0 times 2=1 time 3=2 times 4=3 to 5 times 5=6 to 9 times 6=10 or more times 7=Don't know [mutually exclusive] </t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -2778,7 +2774,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>1=An official institutional communication (e.g., email, emergency alert system) 2=A memorial 3=News media (e.g., newspapers or blogs) 4=Social media (e.g., Reddit, Instagram, Meta, X) 5=Word of mouth from my peers 6=Others  7=I don’t remember 8=None of these</t>
+          <t>1=An official institutional communication (e.g., email, emergency alert system) 2=A memorial 3=News media (e.g., newspapers or blogs) 4=Social media (e.g., Reddit, Instagram, Meta, X) 5=Word of mouth from my peers 6=Others  7=I don’t remember [mutually exclusive] 8=None of these</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -3020,7 +3016,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>1=No negative experience 2=Harassed/Bullied online 3=Cyber stalking 4=Flaming, whereby someone is being encouraged (egged on) to die by suicide 5=Had someone create/share embarrassing images of you using Ai (e.g., deep fakes) 6=Imposter Scam,for falsely demanding money from family and friends 7=Others</t>
+          <t>1=No negative experience [mutually exclusive] 2=Harassed/Bullied online 3=Cyber stalking 4=Flaming, whereby someone is being encouraged (egged on) to die by suicide 5=Had someone create/share embarrassing images of you using Ai (e.g., deep fakes) 6=Imposter Scam,for falsely demanding money from family and friends 7=Others</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -3196,7 +3192,7 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1=Depression (e.g., major depressive disorder, persistent depressive disorder) 2=Bipolar (e.g., bipolar I or II, cyclothymia) 3=Anxiety (e.g., generalized anxiety disorder, phobias) 4=Obsessive-compulsive or related disorders (e.g., obsessive-compulsive disorder, body dysmorphia) 5=Trauma and Stressor Related Disorders (e.g, post-traumatic stress disorder), 6=Neurodevelopmental disorder or intellectual disability (e.g., attention deficit disorder (ADD), attention deficit hyperactivity disorder (ADHD), intellectual disability, autism spectrum disorder) 7=Eating disorder (e.g., anorexia nervosa, bulimia nervosa) 8=Psychosis (e.g., schizophrenia, schizo-affective disorder) 9=Personality disorder (e.g., antisocial personality disorder, paranoid personality disorder, schizoid personality disorder) 10=Substance use disorder (e.g., alcohol abuse, abuse of other drugs) 11=No, none of these [mutually exclusive] 12=Don’t know 13=Other mental health condition (please specify)</t>
+          <t>1=Depression (e.g., major depressive disorder, persistent depressive disorder) 2=Bipolar (e.g., bipolar I or II, cyclothymia) 3=Anxiety (e.g., generalized anxiety disorder, phobias) 4=Obsessive-compulsive or related disorders (e.g., obsessive-compulsive disorder, body dysmorphia) 5=Trauma and Stressor Related Disorders (e.g, post-traumatic stress disorder), 6=Neurodevelopmental disorder or intellectual disability (e.g., attention deficit disorder (ADD), attention deficit hyperactivity disorder (ADHD), intellectual disability, autism spectrum disorder) 7=Eating disorder (e.g., anorexia nervosa, bulimia nervosa) 8=Psychosis (e.g., schizophrenia, schizo-affective disorder) 9=Personality disorder (e.g., antisocial personality disorder, paranoid personality disorder, schizoid personality disorder) 10=Substance use disorder (e.g., alcohol abuse, abuse of other drugs) 11=No, none of these [mutually exclusive] 12=Don't know [mutually exclusive] 13=Other mental health condition (please specify)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -3272,7 +3268,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1=Major depressive disorder 2=Dysthymia or persistent depressive disorder 3=Premenstrual dysphoric disorder 4=Others  5=Don’t know</t>
+          <t>1=Major depressive disorder 2=Dysthymia or persistent depressive disorder 3=Premenstrual dysphoric disorder 4=Others  5=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -3326,7 +3322,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1=Bipolar I disorder 2=Bipolar II disorder 3=Cyclothymic disorder 4=Others  5=Don’t know</t>
+          <t>1=Bipolar I disorder 2=Bipolar II disorder 3=Cyclothymic disorder 4=Others  5=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -3380,7 +3376,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1 =Generalized anxiety disorder 2=Panic disorder 3=Agoraphobia 4=Specific phobia (e.g., claustrophobia, arachnophobia, etc.) 5=Social anxiety disorder (or social phobia) 6=Others  7=Don’t know</t>
+          <t>1 =Generalized anxiety disorder 2=Panic disorder 3=Agoraphobia 4=Specific phobia (e.g., claustrophobia, arachnophobia, etc.) 5=Social anxiety disorder (or social phobia) 6=Others  7=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3434,7 +3430,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1=Obsessive-compulsive disorder 2=Body dysmorphic disorder 3=Hoarding disorder 4=Trichotillomania (hair-pulling disorder) 5=Excoriation (skin-picking) disorder 6=Others 7=Don’t know</t>
+          <t>1=Obsessive-compulsive disorder 2=Body dysmorphic disorder 3=Hoarding disorder 4=Trichotillomania (hair-pulling disorder) 5=Excoriation (skin-picking) disorder 6=Others 7=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3488,7 +3484,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1=Post-traumatic stress disorder 2=Acute stress disorder 3=Adjustment disorder 4=Others  5=Don’t know</t>
+          <t>1=Post-traumatic stress disorder 2=Acute stress disorder 3=Adjustment disorder 4=Others  5=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3542,7 +3538,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1=Attention deficit hyperactivity disorder (ADHD or ADD) 2=Other intellectual disability 3=Autism spectrum disorder 4=Others  5=Don’t know</t>
+          <t>1=Attention deficit hyperactivity disorder (ADHD or ADD) 2=Other intellectual disability 3=Autism spectrum disorder 4=Others  5=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3596,7 +3592,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1=Anorexia nervosa 2=Bulimia nervosa 3=Binge-eating disorder 4=Pica 5=Avoidant/restrictive food intake disorder (selective eating disorder) 6=Others 7=Don’t know</t>
+          <t>1=Anorexia nervosa 2=Bulimia nervosa 3=Binge-eating disorder 4=Pica 5=Avoidant/restrictive food intake disorder (selective eating disorder) 6=Others 7=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3650,7 +3646,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1=Schizophrenia 2=Schizo-affective disorder 3=Brief psychotic disorder 4=Delusional disorder 5=Schizophreniform disorder 6=Others  7=Don’t know</t>
+          <t>1=Schizophrenia 2=Schizo-affective disorder 3=Brief psychotic disorder 4=Delusional disorder 5=Schizophreniform disorder 6=Others  7=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3704,7 +3700,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1=Antisocial personality disorder 2=Avoidant personality disorder 3=Borderline personality disorder 4=Dependent personality disorder 5=Histrionic personality disorder 6=Narcissistic personality disorder 7=Obsessive-Compulsive personality disorder 8=Paranoid personality disorder 9=Schizoid personality disorder 10=Schizotypal personality disorder 11=Others 12=Don’t know</t>
+          <t>1=Antisocial personality disorder 2=Avoidant personality disorder 3=Borderline personality disorder 4=Dependent personality disorder 5=Histrionic personality disorder 6=Narcissistic personality disorder 7=Obsessive-Compulsive personality disorder 8=Paranoid personality disorder 9=Schizoid personality disorder 10=Schizotypal personality disorder 11=Others 12=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3758,7 +3754,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1=Alcohol abuse or other alcohol-related disorders 4=Opioid Use Disorder 2=Others  3=Don’t know</t>
+          <t>1=Alcohol abuse or other alcohol-related disorders 4=Opioid Use Disorder 2=Others  3=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -4962,7 +4958,7 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1=Psychostimulants (methylphenidate, amphetamine salts), dextroamphetamine, etc.) 2=Antidepressants (e.g., fluoxetin,sertraline,paroxetine,escitalopra,venlafaxine,bupropion, etc.) 3=Antipsychotics (e.g., haloperidol,clozapine,risperidone,olanzapine,etc.) 4=Anti-anxiety medications (e.g., lorazepam,clonazepam,alprazolam,buspirone,etc.) 5=Mood stabilizers (e.g., lithium, valproate,lamotrigine,carbamazepine,etc.) 6=Sleep medications (e.g., zolpidem,zaleplon,etc.) 7=Others  8=No, none of these [mutually exclusive] 9=Don’t know</t>
+          <t>1=Psychostimulants (methylphenidate, amphetamine salts), dextroamphetamine, etc.) 2=Antidepressants (e.g., fluoxetin,sertraline,paroxetine,escitalopra,venlafaxine,bupropion, etc.) 3=Antipsychotics (e.g., haloperidol,clozapine,risperidone,olanzapine,etc.) 4=Anti-anxiety medications (e.g., lorazepam,clonazepam,alprazolam,buspirone,etc.) 5=Mood stabilizers (e.g., lithium, valproate,lamotrigine,carbamazepine,etc.) 6=Sleep medications (e.g., zolpidem,zaleplon,etc.) 7=Others  8=No, none of these [mutually exclusive] 9=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -4971,7 +4967,7 @@
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>1.39</v>
+        <v>0</v>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
@@ -5002,11 +4998,11 @@
         </is>
       </c>
       <c r="O32" s="2" t="n">
-        <v>0.597</v>
+        <v>0.6</v>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr"/>
@@ -5146,7 +5142,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1=Not at all 2=1-2 times 3=3-5 times 4=More than 5 times 5=Don’t know</t>
+          <t>1=Not at all 2=1-2 times 3=3-5 times 4=More than 5 times 5=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -5200,7 +5196,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>1=A general practitioner, nurse practitioner, or primary care physician 2=A psychiatrist 3=Other type of doctor  4=Took the medication(s) without a prescription 5=Don’t know</t>
+          <t>1=A general practitioner, nurse practitioner, or primary care physician 2=A psychiatrist 3=Other type of doctor  4=Took the medication(s) without a prescription 5=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -5254,7 +5250,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>1=Psychostimulants (methylphenidate, amphetamine salts), dextroamphetamine, etc.) 2=Antidepressants (e.g., fluoxetin,sertraline,paroxetine,escitalopra,venlafaxine,bupropion, etc.) 3=Antipsychotics (e.g., haloperidol,clozapine,risperidone,olanzapine,etc.) 4=Anti-anxiety medications (e.g., lorazepam,clonazepam,alprazolam,buspirone,etc.) 5=Mood stabilizers (e.g., lithium, valproate,lamotrigine,carbamazepine,etc.) 6=Sleep medications (e.g., zolpidem,zaleplon,etc.) 7=Others  8=No, none of these [mutually exclusive] 9=Don’t know</t>
+          <t>1=Psychostimulants (methylphenidate, amphetamine salts), dextroamphetamine, etc.) 2=Antidepressants (e.g., fluoxetin,sertraline,paroxetine,escitalopra,venlafaxine,bupropion, etc.) 3=Antipsychotics (e.g., haloperidol,clozapine,risperidone,olanzapine,etc.) 4=Anti-anxiety medications (e.g., lorazepam,clonazepam,alprazolam,buspirone,etc.) 5=Mood stabilizers (e.g., lithium, valproate,lamotrigine,carbamazepine,etc.) 6=Sleep medications (e.g., zolpidem,zaleplon,etc.) 7=Others  8=No, none of these [mutually exclusive] 9=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -5617,7 +5613,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Which of the following are important reasons why you received the counselling services? (Select all that apply)</t>
+          <t>Which of the following are important reasons why you received those services? (Select all that apply)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -6594,7 +6590,7 @@
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1=Diabetes 2=High blood pressure 3=Asthma 4=Thyroid disease (e.g., hypothyroid or hyperthyroid) 5=Gastrointestinal disease (e.g., Crohn’s Disease, Ulcerative Colitis) 6=Arthritis 7=Sickle cell anemia 8=Seizure disorders (e.g., epilepsy) 9=Cancers 10=High cholesterol 11=HIV/AIDS 12=Other autoimmune disorder  13=Other chronic disease  14=No, never been diagnosed with a chronic disease. [mutually exclusive] 15=Don’t know [mutually exclusive]</t>
+          <t>1=Diabetes 2=High blood pressure 3=Asthma 4=Thyroid disease (e.g., hypothyroid or hyperthyroid) 5=Gastrointestinal disease (e.g., Crohn’s Disease, Ulcerative Colitis) 6=Arthritis 7=Sickle cell anemia 8=Seizure disorders (e.g., epilepsy) 9=Cancers 10=High cholesterol 11=HIV/AIDS 12=Other autoimmune disorder  13=Other chronic disease  14=No, never been diagnosed with a chronic disease. [mutually exclusive] 15=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -6864,7 +6860,7 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>0=No 1=Yes 2=I don’t know 3=Prefer not to say</t>
+          <t>0=No 1=Yes 2=I Don't know [mutually exclusive] 3=Prefer not to say</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -6873,11 +6869,11 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>77.33</v>
+        <v>67.77</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -6904,7 +6900,7 @@
         </is>
       </c>
       <c r="O7" s="2" t="n">
-        <v>0.212</v>
+        <v>0.231</v>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -6936,7 +6932,7 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>0=No 1=Yes 2=I don’t know 3=Prefer not to say</t>
+          <t>0=No 1=Yes 2=I Don't know [mutually exclusive] 3=Prefer not to say</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -6945,11 +6941,11 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>75.44</v>
+        <v>67.16</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -6976,7 +6972,7 @@
         </is>
       </c>
       <c r="O8" s="2" t="n">
-        <v>0.216</v>
+        <v>0.232</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -7066,7 +7062,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1=Less than 5 minutes 2=Between 5 and 30 minutes 3=More than 30 minutes but less than 24 hours 4=24 hours or longer 5=I don’t know 6=Prefer not to say</t>
+          <t>1=Less than 5 minutes 2=Between 5 and 30 minutes 3=More than 30 minutes but less than 24 hours 4=24 hours or longer 5=I Don't know [mutually exclusive] 6=Prefer not to say</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -8237,7 +8233,7 @@
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>1=2-year college degree (associate’s) 2=4-year college degree (bachelor’s) 3=Master’s degree 4=Doctoral degree (JD, MD, Ph D, etc.) 5=Other degree  6=Don’t know</t>
+          <t>1=2-year college degree (associate’s) 2=4-year college degree (bachelor’s) 3=Master’s degree 4=Doctoral degree (JD, MD, Ph D, etc.) 5=Other degree  6=Don't know [mutually exclusive]</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -8246,7 +8242,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68.31999999999999</v>
+        <v>59.53</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -8277,7 +8273,7 @@
         </is>
       </c>
       <c r="O9" s="2" t="n">
-        <v>0.063</v>
+        <v>0.081</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
dry run fix #4
</commit_message>
<xml_diff>
--- a/SurveyQuestions/outputs/hms_question_score.xlsx
+++ b/SurveyQuestions/outputs/hms_question_score.xlsx
@@ -1627,7 +1627,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Please answer the following questions as honestly as possible. 1. Do you often feel the desire to eat when you are emotionally upset or stressed? 2. Do you often feel that you can't control what or how much you eat? 3. Do you sometimes make yourself throw up (vomit) to control your weight? 4. Are you often preoccupied with a desire to be thinner? 5. Do you believe yourself to be fat when others say you are thin?</t>
+          <t>Please answer the following questions as honestly as possible.
+1. Do you often feel the desire to eat when you are emotionally upset or stressed?
+2. Do you often feel that you can't control what or how much you eat?
+3. Do you sometimes make yourself throw up (vomit) to control your weight?
+4. Are you often preoccupied with a desire to be thinner?
+5. Do you believe yourself to be fat when others say you are thin?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3001,7 +3006,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>We know that there are many experiences in the online space, ranging from positive to neutral to negative. For this item, we want to know more about your negative online experiences. Please select all the negative experiences you have had in online spaces (such as social media) in the past year.</t>
+          <t>We know that there are many experiences in the online space, ranging from positive to neutral to negative. For this item, we want to know more about your negative online experiences. Please select all the negative experiences you have had in online spaces (such as social media) in the past year. (Select all that apply)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
dry run fix #5
</commit_message>
<xml_diff>
--- a/SurveyQuestions/outputs/hms_question_score.xlsx
+++ b/SurveyQuestions/outputs/hms_question_score.xlsx
@@ -1795,7 +1795,7 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>1=Cut myself 2=Burned myself 3=Punched or banged myself 4=Scratched myself 5=Pulled my hair 6=Bit myself 7=Interfered with wound healing 8=Carved words or symbols into skin 9=Rubbed sharp objects into skin 10=Punched or banged an object to hurt myself 11=Other (please specify) 12=No, none of these [mutually exclusive]</t>
+          <t>1=Cut myself 2=Burned myself 3=Punched or banged myself 4=Scratched myself 5=Pulled my hair 6=Bit myself 7=Interfered with wound healing 8=Carved words or symbols into skin 9=Rubbed sharp objects into skin 10=Punched or banged an object to hurt myself 11=Others 12=No, none of these [mutually exclusive]</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1804,7 +1804,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>59.75</v>
+        <v>61.88</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="O12" s="2" t="n">
-        <v>0.481</v>
+        <v>0.476</v>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>

</xml_diff>